<commit_message>
Big change to modify for error
</commit_message>
<xml_diff>
--- a/test/RQ2_test/Ablation/rq2_ablation_result.xlsx
+++ b/test/RQ2_test/Ablation/rq2_ablation_result.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\29737\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824CEB61-DED0-4A47-816A-4DA98CCD9874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C78CAAE-B7BD-43A7-AFF0-CDB95A027AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="310" yWindow="2220" windowWidth="13980" windowHeight="12560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11290" yWindow="2320" windowWidth="12470" windowHeight="12420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3625,5 +3620,6 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>